<commit_message>
Add payment type (AQ) to PAID/NOT PAID/TROUBLE comments in МЕТЕОР orders
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Orders_МЕТЕОР_filled.xlsx
+++ b/output/Orders_МЕТЕОР_filled.xlsx
@@ -656,7 +656,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2 PAID</t>
+          <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1 NOT PAID</t>
+          <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1 NOT PAID</t>
+          <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1 NOT PAID</t>
+          <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1 NOT PAID</t>
+          <t>1 NOT PAID, тип оплаты: Постоплата 100%</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2 PAID</t>
+          <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>6 TROUBLE</t>
+          <t>6 TROUBLE, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2 PAID</t>
+          <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2 PAID</t>
+          <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>1 NOT PAID</t>
+          <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1 NOT PAID</t>
+          <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2 PAID</t>
+          <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preserve original formatting in МЕТЕОР orders file
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Orders_МЕТЕОР_filled.xlsx
+++ b/output/Orders_МЕТЕОР_filled.xlsx
@@ -2,26 +2,56 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25420" windowHeight="16300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Резиденты" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="122211" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color rgb="FF3F4350"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color indexed="81"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -34,7 +64,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,17 +72,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -125,9 +178,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -165,7 +218,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -199,6 +252,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -233,9 +287,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -414,1021 +469,1082 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="12.453125" customWidth="1" min="1" max="1"/>
+    <col width="40.54296875" customWidth="1" min="2" max="2"/>
+    <col width="13.81640625" customWidth="1" min="3" max="3"/>
+    <col width="12.1796875" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="11.26953125" customWidth="1" min="7" max="7"/>
+    <col width="12.1796875" customWidth="1" min="8" max="8"/>
+    <col width="15.26953125" customWidth="1" min="9" max="9"/>
+    <col width="15.54296875" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="14.5" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Order №</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Order State</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Detail State</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Part No</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Backorder</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Target date </t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Confirmed date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="14.5" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>P19105026</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>BMS13-65T0G</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>23.02.2026</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>01.04.2026</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>7 REFUND</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="14.5" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>P19994326</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>10-60806-7</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="F3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>04.07.2026</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>14.07.2026</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>Не найдено в ТАЗ</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="14.5" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>P19907626</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>PARTLY RECEIVED</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>BACB30MY6K10</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>10.07.2026</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>25.07.2026</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="1" t="inlineStr">
         <is>
           <t>Отгружен 20.06.2026</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="14.5" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>P20056426</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>G7500-03</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="F5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>19.07.2026</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>03.08.2026</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="1" t="inlineStr">
         <is>
           <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="14.5" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>P19557226</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>0YX1600A04G01</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="F6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>16.05.2026</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>04.08.2026</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="1" t="inlineStr">
         <is>
           <t>Отгружен 10.06.2026</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="14.5" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>P19569126</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>898732-02</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="F7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
         <is>
           <t>08.05.2026</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="1" t="inlineStr">
         <is>
           <t>04.08.2026</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="1" t="inlineStr">
         <is>
           <t>Отгружен 06.06.2026</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="14.5" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>P20065826</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>02-190002-018</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="1" t="inlineStr">
         <is>
           <t>30.07.2026</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="1" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="1" t="inlineStr">
         <is>
           <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="14.5" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>P20065826</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>02-190002-020</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="1" t="inlineStr">
         <is>
           <t>30.07.2026</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="1" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="1" t="inlineStr">
         <is>
           <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="14.5" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>P20065826</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>06-133802-002</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="F10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
         <is>
           <t>29.07.2026</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="1" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="1" t="inlineStr">
         <is>
           <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="14.5" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>P20189826</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>BACB30NX12K20</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>13.07.2026</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="1" t="inlineStr">
         <is>
           <t>1 NOT PAID, тип оплаты: Постоплата 100%</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="14.5" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>P20004326</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>2-230S604-70</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="1" t="inlineStr">
         <is>
           <t>20.07.2026</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="1" t="inlineStr">
         <is>
           <t>09.08.2026</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="1" t="inlineStr">
         <is>
           <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="13" ht="14.5" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>P20228326</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>BACC2C4C06720EG</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="F13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>20.07.2026</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="1" t="inlineStr">
         <is>
           <t>09.08.2026</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="1" t="inlineStr">
         <is>
           <t>6 TROUBLE, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="14" ht="14.5" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>P20060126</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>320362-2-1</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="F14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
         <is>
           <t>24.07.2026</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="1" t="inlineStr">
         <is>
           <t>13.08.2026</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="1" t="inlineStr">
         <is>
           <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="15" ht="14.5" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>P20094326</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>3604524-54</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="F15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
         <is>
           <t>30.07.2026</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="1" t="inlineStr">
         <is>
           <t>14.08.2026</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="1" t="inlineStr">
         <is>
           <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="16" ht="14.5" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>P20249926</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>C20633000</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="F16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
         <is>
           <t>07.08.2026</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="1" t="inlineStr">
         <is>
           <t>17.08.2026</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="1" t="inlineStr">
         <is>
           <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="14.5" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>P19915126</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>NAS1149D0332J</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="1" t="inlineStr">
         <is>
           <t>01.07.2026</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="1" t="inlineStr">
         <is>
           <t>19.08.2026</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="1" t="inlineStr">
         <is>
           <t>Отгружен 20.06.2026</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="14.5" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>P19924226</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>MS21083C3</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="1" t="inlineStr">
         <is>
           <t>27.06.2026</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="1" t="inlineStr">
         <is>
           <t>19.08.2026</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="1" t="inlineStr">
         <is>
           <t>Отгружен 20.06.2026</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19" ht="14.5" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>P19943126</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>0LN115-18K</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="1" t="inlineStr">
         <is>
           <t>06.07.2026</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="1" t="inlineStr">
         <is>
           <t>19.08.2026</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="1" t="inlineStr">
         <is>
           <t>Отгружен 20.06.2026</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="20" ht="14.5" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>P19477526</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>2100M96P05</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="1" t="n">
         <v>80</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" s="1" t="n">
         <v>80</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="1" t="inlineStr">
         <is>
           <t>20.08.2026</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="1" t="inlineStr">
         <is>
           <t>20.08.2026</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="1" t="inlineStr">
         <is>
           <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="21" ht="14.5" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>P19863426</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>МЕТЕОР</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>W260F4AM11</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="F21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>18.06.2026</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>21.08.2026</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>2 PAID, тип оплаты: Частичная предоплата</t>
         </is>
       </c>
     </row>
+    <row r="22" ht="14.5" customHeight="1"/>
+    <row r="23" ht="14.5" customHeight="1"/>
+    <row r="24" ht="14.5" customHeight="1"/>
+    <row r="25" ht="14.5" customHeight="1"/>
+    <row r="26" ht="14.5" customHeight="1"/>
+    <row r="27" ht="14.5" customHeight="1"/>
+    <row r="28" ht="14.5" customHeight="1"/>
+    <row r="29" ht="14.5" customHeight="1"/>
+    <row r="30" ht="14.5" customHeight="1"/>
+    <row r="31" ht="14.5" customHeight="1"/>
+    <row r="32" ht="14.5" customHeight="1"/>
+    <row r="33" ht="14.5" customHeight="1"/>
+    <row r="34" ht="14.5" customHeight="1"/>
+    <row r="35" ht="14.5" customHeight="1"/>
+    <row r="36" ht="14.5" customHeight="1"/>
+    <row r="37" ht="14.5" customHeight="1"/>
+    <row r="38" ht="14.5" customHeight="1"/>
+    <row r="39" ht="14.5" customHeight="1"/>
+    <row r="40" ht="14.5" customHeight="1"/>
+    <row r="41" ht="14.5" customHeight="1"/>
+    <row r="42" ht="14.5" customHeight="1"/>
+    <row r="43" ht="14.5" customHeight="1"/>
+    <row r="44" ht="14.5" customHeight="1"/>
+    <row r="45" ht="14.5" customHeight="1"/>
+    <row r="46" ht="14.5" customHeight="1"/>
+    <row r="47" ht="14.5" customHeight="1"/>
+    <row r="48" ht="14.5" customHeight="1"/>
+    <row r="49" ht="14.5" customHeight="1"/>
+    <row r="50" ht="14.5" customHeight="1"/>
+    <row r="51" ht="14.5" customHeight="1"/>
+    <row r="52" ht="14.5" customHeight="1"/>
+    <row r="53" ht="14.5" customHeight="1"/>
+    <row r="54" ht="14.5" customHeight="1"/>
+    <row r="55" ht="14.5" customHeight="1"/>
+    <row r="56" ht="14.5" customHeight="1"/>
+    <row r="57" ht="14.5" customHeight="1"/>
+    <row r="58" ht="14.5" customHeight="1"/>
+    <row r="59" ht="14.5" customHeight="1"/>
+    <row r="60" ht="14.5" customHeight="1"/>
+    <row r="61" ht="14.5" customHeight="1"/>
+    <row r="62" ht="14.5" customHeight="1"/>
+    <row r="63" ht="14.5" customHeight="1"/>
+    <row r="64" ht="14.5" customHeight="1"/>
+    <row r="65" ht="14.5" customHeight="1"/>
+    <row r="66" ht="14.5" customHeight="1"/>
+    <row r="67" ht="14.5" customHeight="1"/>
+    <row r="68" ht="14.5" customHeight="1"/>
+    <row r="69" ht="14.5" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mark unpaid prepayment orders as awaiting advance payment
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Orders_МЕТЕОР_filled.xlsx
+++ b/output/Orders_МЕТЕОР_filled.xlsx
@@ -3,20 +3,20 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25420" windowHeight="16300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7430" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Резиденты" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="122211" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,13 +30,6 @@
       <family val="2"/>
       <color rgb="FF3F4350"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Tahoma"/>
-      <charset val="204"/>
-      <family val="2"/>
-      <color indexed="81"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -95,10 +88,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -472,15 +465,15 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12.453125" customWidth="1" min="1" max="1"/>
-    <col width="40.54296875" customWidth="1" min="2" max="2"/>
+    <col width="10.36328125" customWidth="1" min="2" max="2"/>
     <col width="13.81640625" customWidth="1" min="3" max="3"/>
     <col width="12.1796875" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="16.26953125" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="11.26953125" customWidth="1" min="7" max="7"/>
     <col width="12.1796875" customWidth="1" min="8" max="8"/>
     <col width="15.26953125" customWidth="1" min="9" max="9"/>
-    <col width="15.54296875" customWidth="1" min="10" max="10"/>
+    <col width="50.90625" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.5" customHeight="1">
@@ -579,7 +572,7 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>7 REFUND</t>
+          <t>Заказ отменен 27.03</t>
         </is>
       </c>
     </row>
@@ -627,7 +620,7 @@
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
-          <t>Не найдено в ТАЗ</t>
+          <t>Заказ вами не размещался</t>
         </is>
       </c>
     </row>
@@ -723,7 +716,7 @@
       </c>
       <c r="J5" s="1" t="inlineStr">
         <is>
-          <t>2 PAID, тип оплаты: Частичная предоплата</t>
+          <t>Заказ в работе, ожидаем авансовый платеж</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1052,7 @@
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>2 PAID, тип оплаты: Частичная предоплата</t>
+          <t>Заказ в работе, ожидаем авансовый платеж</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1148,7 @@
       </c>
       <c r="J14" s="1" t="inlineStr">
         <is>
-          <t>2 PAID, тип оплаты: Частичная предоплата</t>
+          <t>Заказ в работе, ожидаем авансовый платеж</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1196,7 @@
       </c>
       <c r="J15" s="1" t="inlineStr">
         <is>
-          <t>2 PAID, тип оплаты: Частичная предоплата</t>
+          <t>Заказ в работе, ожидаем авансовый платеж</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1244,7 @@
       </c>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>1 NOT PAID, тип оплаты: Частичная предоплата</t>
+          <t>Заказ в работе, ожидаем авансовый платеж</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Comments for МЕТЕОР order P20320926
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Orders_МЕТЕОР_filled.xlsx
+++ b/output/Orders_МЕТЕОР_filled.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12.453125" customWidth="1" min="1" max="1"/>
@@ -538,7 +538,7 @@
     <row r="2" ht="14.5" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>P19705326</t>
+          <t>P20320926</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -558,127 +558,33 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>M472001-01</t>
+          <t>R259G11</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>11.06.2026</t>
+          <t>06.08.2026</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>31.08.2026</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Отгружен 31.07.2026</t>
+          <t>Заказ в работе, ожидаем авансовый платеж</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14.5" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>P20065726</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>G7500-03</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>27.07.2026</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>01.08.2026</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>Отгружен 29.07.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="14.5" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>P20150926</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>МЕТЕОР</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>J221P906WE</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>70</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>70</v>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>10.08.2026</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>30.08.2026</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>Заказ в работе, ожидаем авансовый платеж</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="14.5" customHeight="1"/>
+    <row r="4" ht="14.5" customHeight="1"/>
     <row r="5" ht="14.5" customHeight="1"/>
     <row r="6" ht="14.5" customHeight="1"/>
     <row r="7" ht="14.5" customHeight="1"/>
@@ -725,8 +631,6 @@
     <row r="48" ht="14.5" customHeight="1"/>
     <row r="49" ht="14.5" customHeight="1"/>
     <row r="50" ht="14.5" customHeight="1"/>
-    <row r="51" ht="14.5" customHeight="1"/>
-    <row r="52" ht="14.5" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>

</xml_diff>